<commit_message>
augmentaion, power capex, degradation in main
</commit_message>
<xml_diff>
--- a/inputs/bess_installs_capex.xlsx
+++ b/inputs/bess_installs_capex.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f9c6ffa232d49179/Documents/Solar_BESS/inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\barna\PycharmProjects\solar_bess\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="240" documentId="8_{2B54CD34-4F41-4A71-BD30-FFDF0095B63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE3343BE-7A40-434C-8F0B-7286608AF0BB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58918E2C-AE97-4EAA-82AA-01F6EE5C5DC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B92BE577-E5A6-49BC-BFF6-C9C17C524DC8}"/>
+    <workbookView xWindow="17550" yWindow="-13995" windowWidth="20760" windowHeight="12390" xr2:uid="{B92BE577-E5A6-49BC-BFF6-C9C17C524DC8}"/>
   </bookViews>
   <sheets>
     <sheet name="battery_kwh" sheetId="2" r:id="rId1"/>

</xml_diff>